<commit_message>
H40: amplitud en px del mismo grupo que el %
</commit_message>
<xml_diff>
--- a/data/processed_data/Video_prueba/contracciones_Video_prueba.xlsx
+++ b/data/processed_data/Video_prueba/contracciones_Video_prueba.xlsx
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V4"/>
+  <dimension ref="A1:W4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -811,85 +811,90 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>amplitud_px</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>ttp_n_eventos</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>ttp_n_medibles</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>ttp_frames_mediana</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>ttp_reportable</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>ttp_s</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>ttp_iqr_s</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>ttp_cota_inf_s</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>ttp_cota_sup_s</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>rt50_n_eventos</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>rt50_n_medibles</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>rt50_frames_mediana</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>rt50_reportable</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>rt50_s</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>rt50_iqr_s</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>rt50_cota_inf_s</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>rt50_cota_sup_s</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>cinetica_motivo</t>
         </is>
@@ -916,46 +921,49 @@
         </is>
       </c>
       <c r="F2" t="n">
+        <v>2.093700000000013</v>
+      </c>
+      <c r="G2" t="n">
         <v>29</v>
       </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
       <c r="H2" t="n">
-        <v>2</v>
-      </c>
-      <c r="I2" t="b">
-        <v>0</v>
-      </c>
-      <c r="J2" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J2" t="b">
+        <v>0</v>
+      </c>
       <c r="K2" t="inlineStr"/>
-      <c r="L2" t="n">
-        <v>0</v>
-      </c>
+      <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="n">
         <v>0.1016666666666666</v>
       </c>
-      <c r="N2" t="n">
+      <c r="O2" t="n">
         <v>29</v>
       </c>
-      <c r="O2" t="n">
-        <v>0</v>
-      </c>
       <c r="P2" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R2" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>2</v>
+      </c>
+      <c r="R2" t="b">
+        <v>0</v>
+      </c>
       <c r="S2" t="inlineStr"/>
-      <c r="T2" t="n">
-        <v>0</v>
-      </c>
+      <c r="T2" t="inlineStr"/>
       <c r="U2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V2" t="n">
         <v>0.1016666666666683</v>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>TTP: medible en 0 de 29 eventos (&lt; la mitad con &gt;= 5 fotogramas); solo cota TTP &lt; 102 ms; RT50: medible en 0 de 29 eventos (&lt; la mitad con &gt;= 5 fotogramas); solo cota RT50 &lt; 102 ms</t>
         </is>
@@ -982,46 +990,49 @@
         </is>
       </c>
       <c r="F3" t="n">
+        <v>6.807450000000017</v>
+      </c>
+      <c r="G3" t="n">
         <v>6</v>
       </c>
-      <c r="G3" t="n">
-        <v>0</v>
-      </c>
       <c r="H3" t="n">
-        <v>2</v>
-      </c>
-      <c r="I3" t="b">
-        <v>0</v>
-      </c>
-      <c r="J3" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J3" t="b">
+        <v>0</v>
+      </c>
       <c r="K3" t="inlineStr"/>
-      <c r="L3" t="n">
-        <v>0</v>
-      </c>
+      <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="n">
         <v>0.1008333333333331</v>
       </c>
-      <c r="N3" t="n">
+      <c r="O3" t="n">
         <v>6</v>
       </c>
-      <c r="O3" t="n">
-        <v>0</v>
-      </c>
       <c r="P3" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q3" t="b">
-        <v>0</v>
-      </c>
-      <c r="R3" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>2</v>
+      </c>
+      <c r="R3" t="b">
+        <v>0</v>
+      </c>
       <c r="S3" t="inlineStr"/>
-      <c r="T3" t="n">
-        <v>0</v>
-      </c>
+      <c r="T3" t="inlineStr"/>
       <c r="U3" t="n">
+        <v>0</v>
+      </c>
+      <c r="V3" t="n">
         <v>0.1008333333333304</v>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>TTP: medible en 0 de 6 eventos (&lt; la mitad con &gt;= 5 fotogramas); solo cota TTP &lt; 101 ms; RT50: medible en 0 de 6 eventos (&lt; la mitad con &gt;= 5 fotogramas); solo cota RT50 &lt; 101 ms</t>
         </is>
@@ -1048,46 +1059,49 @@
         </is>
       </c>
       <c r="F4" t="n">
+        <v>2.07185000000004</v>
+      </c>
+      <c r="G4" t="n">
         <v>23</v>
       </c>
-      <c r="G4" t="n">
-        <v>0</v>
-      </c>
       <c r="H4" t="n">
-        <v>2</v>
-      </c>
-      <c r="I4" t="b">
-        <v>0</v>
-      </c>
-      <c r="J4" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J4" t="b">
+        <v>0</v>
+      </c>
       <c r="K4" t="inlineStr"/>
-      <c r="L4" t="n">
-        <v>0</v>
-      </c>
+      <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
         <v>0.1016666666666666</v>
       </c>
-      <c r="N4" t="n">
+      <c r="O4" t="n">
         <v>23</v>
       </c>
-      <c r="O4" t="n">
-        <v>0</v>
-      </c>
       <c r="P4" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q4" t="b">
-        <v>0</v>
-      </c>
-      <c r="R4" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>2</v>
+      </c>
+      <c r="R4" t="b">
+        <v>0</v>
+      </c>
       <c r="S4" t="inlineStr"/>
-      <c r="T4" t="n">
-        <v>0</v>
-      </c>
+      <c r="T4" t="inlineStr"/>
       <c r="U4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V4" t="n">
         <v>0.1033333333333335</v>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t>TTP: medible en 0 de 23 eventos (&lt; la mitad con &gt;= 5 fotogramas); solo cota TTP &lt; 102 ms; RT50: medible en 0 de 23 eventos (&lt; la mitad con &gt;= 5 fotogramas); solo cota RT50 &lt; 103 ms</t>
         </is>
@@ -1104,7 +1118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BL2"/>
+  <dimension ref="A1:BM2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1270,160 +1284,165 @@
       </c>
       <c r="AG1" t="inlineStr">
         <is>
+          <t>amplitud_px</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
           <t>ttp_n_eventos</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>ttp_n_medibles</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>ttp_frames_mediana</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>ttp_reportable</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>ttp_s</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>ttp_iqr_s</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>ttp_cota_inf_s</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>ttp_cota_sup_s</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>rt50_n_eventos</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>rt50_n_medibles</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>rt50_frames_mediana</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>rt50_reportable</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>rt50_s</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>rt50_iqr_s</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>rt50_cota_inf_s</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>rt50_cota_sup_s</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>cinetica_motivo</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>fotogramas_sin_medida</t>
         </is>
       </c>
-      <c r="AY1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>fotogramas_sin_medida_pct</t>
         </is>
       </c>
-      <c r="AZ1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
         <is>
           <t>fotogramas_low_quality</t>
         </is>
       </c>
-      <c r="BA1" t="inlineStr">
+      <c r="BB1" t="inlineStr">
         <is>
           <t>eventos_junto_a_hueco</t>
         </is>
       </c>
-      <c r="BB1" t="inlineStr">
+      <c r="BC1" t="inlineStr">
         <is>
           <t>eventos_junto_al_borde</t>
         </is>
       </c>
-      <c r="BC1" t="inlineStr">
+      <c r="BD1" t="inlineStr">
         <is>
           <t>win_s_usado</t>
         </is>
       </c>
-      <c r="BD1" t="inlineStr">
+      <c r="BE1" t="inlineStr">
         <is>
           <t>win_s_automatico</t>
         </is>
       </c>
-      <c r="BE1" t="inlineStr">
+      <c r="BF1" t="inlineStr">
         <is>
           <t>duracion_evento_max_s</t>
         </is>
       </c>
-      <c r="BF1" t="inlineStr">
+      <c r="BG1" t="inlineStr">
         <is>
           <t>ventana_corta</t>
         </is>
       </c>
-      <c r="BG1" t="inlineStr">
+      <c r="BH1" t="inlineStr">
         <is>
           <t>conteo_por_ventana</t>
         </is>
       </c>
-      <c r="BH1" t="inlineStr">
+      <c r="BI1" t="inlineStr">
         <is>
           <t>conteo_estable_ventana</t>
         </is>
       </c>
-      <c r="BI1" t="inlineStr">
+      <c r="BJ1" t="inlineStr">
         <is>
           <t>mesetas</t>
         </is>
       </c>
-      <c r="BJ1" t="inlineStr">
+      <c r="BK1" t="inlineStr">
         <is>
           <t>ruido_borde_sup_px</t>
         </is>
       </c>
-      <c r="BK1" t="inlineStr">
+      <c r="BL1" t="inlineStr">
         <is>
           <t>ruido_borde_inf_px</t>
         </is>
       </c>
-      <c r="BL1" t="inlineStr">
+      <c r="BM1" t="inlineStr">
         <is>
           <t>cociente_ruido_bordes</t>
         </is>
@@ -1500,9 +1519,9 @@
        'estimulados', 'estimulados', 'estimulados', 'estimulados',
        'estimulados'], dtype=object), 'tren_por_evento': array([0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 1, 0, 0,
        0, 0, 1, 1, 1, 1, 1]), 'estimulados': array([19, 24, 25, 26, 27, 28]), 'estimulados_dudosos': array([], dtype=int64), 'espontaneos': array([ 0,  1,  2,  3,  4,  5,  6,  7,  8,  9, 10, 11, 12, 13, 14, 15, 16,
-       17, 18, 20, 21, 22, 23]), 'hay_estimulacion': True, 'n_trenes_estimulados': 1, 'tren_principal': 1, 'veredicto': 'enganchado a la frecuencia configurada (0.1 Hz)', 'z': 17.248, 'p_valor': 0.000999000999000999, 'periodo_grilla_s': 9.9682, 'periodo_s': 10.00043, 'periodo_err_s': 0.0023, 'frecuencia_Hz': 0.1, 'frecuencia_err_Hz': 2.3e-05, 'jitter_s': np.float64(0.00962), 'tolerancia_s': 0.0667, 'n_estimulados': 6, 'n_ranuras': 6, 'tasa_captura_pct': 100.0, 'tren_inicio_s': 14.875, 'tren_fin_s': 64.875, 'jitter_limitado_por_resolucion': True, 'resumen_grupos':          grupo   n  ...  amplitud_mediana_px  amplitud_IQR_px
-0  estimulados   6  ...               6.8075           0.2705
-1  espontaneos  23  ...               2.0719           0.1889
+       17, 18, 20, 21, 22, 23]), 'hay_estimulacion': True, 'n_trenes_estimulados': 1, 'tren_principal': 1, 'veredicto': 'enganchado a la frecuencia configurada (0.1 Hz)', 'z': 17.248, 'p_valor': 0.000999000999000999, 'periodo_grilla_s': 9.9682, 'periodo_s': 10.00043, 'periodo_err_s': 0.0023, 'frecuencia_Hz': 0.1, 'frecuencia_err_Hz': 2.3e-05, 'jitter_s': np.float64(0.00962), 'tolerancia_s': 0.0667, 'n_estimulados': 6, 'n_ranuras': 6, 'tasa_captura_pct': 100.0, 'tren_inicio_s': 14.875, 'tren_fin_s': 64.875, 'jitter_limitado_por_resolucion': True, 'resumen_grupos':          grupo   n  t_inicio_s  ...  CV_intervalo_pct  amplitud_mediana_px  amplitud_IQR_px
+0  estimulados   6       14.87  ...               0.0               6.8075           0.2705
+1  espontaneos  23        0.28  ...              90.6               2.0719           0.1889
 [2 rows x 10 columns], 'espontaneas_instantanea':     tiempo_s  intervalo_s  frecuencia_Hz
 0      0.569       0.5813         1.7204
 1      1.139       0.5593         1.7880
@@ -1584,53 +1603,53 @@
         </is>
       </c>
       <c r="AG2" t="n">
+        <v>6.807450000000017</v>
+      </c>
+      <c r="AH2" t="n">
         <v>6</v>
       </c>
-      <c r="AH2" t="n">
-        <v>0</v>
-      </c>
       <c r="AI2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AJ2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK2" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AK2" t="b">
+        <v>0</v>
+      </c>
       <c r="AL2" t="inlineStr"/>
-      <c r="AM2" t="n">
-        <v>0</v>
-      </c>
+      <c r="AM2" t="inlineStr"/>
       <c r="AN2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO2" t="n">
         <v>0.1008333333333331</v>
       </c>
-      <c r="AO2" t="n">
+      <c r="AP2" t="n">
         <v>6</v>
       </c>
-      <c r="AP2" t="n">
-        <v>0</v>
-      </c>
       <c r="AQ2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AR2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AS2" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS2" t="b">
+        <v>0</v>
+      </c>
       <c r="AT2" t="inlineStr"/>
-      <c r="AU2" t="n">
-        <v>0</v>
-      </c>
+      <c r="AU2" t="inlineStr"/>
       <c r="AV2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW2" t="n">
         <v>0.1008333333333304</v>
       </c>
-      <c r="AW2" t="inlineStr">
+      <c r="AX2" t="inlineStr">
         <is>
           <t>TTP: medible en 0 de 6 eventos (&lt; la mitad con &gt;= 5 fotogramas); solo cota TTP &lt; 101 ms; RT50: medible en 0 de 6 eventos (&lt; la mitad con &gt;= 5 fotogramas); solo cota RT50 &lt; 101 ms</t>
         </is>
       </c>
-      <c r="AX2" t="n">
-        <v>0</v>
-      </c>
       <c r="AY2" t="n">
         <v>0</v>
       </c>
@@ -1641,40 +1660,43 @@
         <v>0</v>
       </c>
       <c r="BB2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BC2" t="n">
         <v>2</v>
       </c>
-      <c r="BD2" t="b">
-        <v>1</v>
-      </c>
-      <c r="BE2" t="n">
+      <c r="BD2" t="n">
+        <v>2</v>
+      </c>
+      <c r="BE2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BF2" t="n">
         <v>0.2333333333333201</v>
       </c>
-      <c r="BF2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BG2" t="inlineStr">
+      <c r="BG2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BH2" t="inlineStr">
         <is>
           <t>1.5 s: 29 | 2 s: 29 | 3 s: 29</t>
         </is>
       </c>
-      <c r="BH2" t="b">
-        <v>1</v>
-      </c>
-      <c r="BI2" t="inlineStr">
+      <c r="BI2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BJ2" t="inlineStr">
         <is>
           <t>29 ev en k=5.315-15.163</t>
         </is>
       </c>
-      <c r="BJ2" t="n">
+      <c r="BK2" t="n">
         <v>0.1095641400000554</v>
       </c>
-      <c r="BK2" t="n">
+      <c r="BL2" t="n">
         <v>0.08569428000006364</v>
       </c>
-      <c r="BL2" t="n">
+      <c r="BM2" t="n">
         <v>1.278546712802465</v>
       </c>
     </row>

</xml_diff>